<commit_message>
Separate BOM generated #4
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Bill of Materials-John_Main.xlsx
+++ b/Deliverables/BOM/Bill of Materials-John_Main.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\JohnWollam-MatrixProject\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\JohnWollam-MatrixProject\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{125E2DA5-DCC7-4888-879A-660E0F4D49B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -944,7 +943,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -1845,6 +1844,15 @@
     <xf numFmtId="0" fontId="20" fillId="4" borderId="21" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
@@ -1872,15 +1880,6 @@
     <xf numFmtId="0" fontId="21" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2217,7 +2216,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:U61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2249,8 +2248,8 @@
       <c r="G1" s="30"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="111"/>
-      <c r="K1" s="112"/>
+      <c r="J1" s="104"/>
+      <c r="K1" s="105"/>
       <c r="L1" s="18"/>
       <c r="M1" s="18"/>
     </row>
@@ -2278,8 +2277,8 @@
       <c r="Q2" s="10"/>
       <c r="R2" s="10"/>
       <c r="S2" s="10"/>
-      <c r="T2" s="107"/>
-      <c r="U2" s="108"/>
+      <c r="T2" s="110"/>
+      <c r="U2" s="111"/>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2306,7 +2305,7 @@
       <c r="R3" s="4"/>
       <c r="S3" s="4"/>
       <c r="T3" s="4"/>
-      <c r="U3" s="105"/>
+      <c r="U3" s="108"/>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2333,7 +2332,7 @@
       <c r="R4" s="4"/>
       <c r="S4" s="4"/>
       <c r="T4" s="4"/>
-      <c r="U4" s="106"/>
+      <c r="U4" s="109"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2360,7 +2359,7 @@
       <c r="R5" s="4"/>
       <c r="S5" s="4"/>
       <c r="T5" s="4"/>
-      <c r="U5" s="106"/>
+      <c r="U5" s="109"/>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2383,7 +2382,7 @@
       <c r="R6" s="4"/>
       <c r="S6" s="4"/>
       <c r="T6" s="4"/>
-      <c r="U6" s="106"/>
+      <c r="U6" s="109"/>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2406,7 +2405,7 @@
       <c r="R7" s="4"/>
       <c r="S7" s="4"/>
       <c r="T7" s="4"/>
-      <c r="U7" s="106"/>
+      <c r="U7" s="109"/>
     </row>
     <row r="8" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2429,7 +2428,7 @@
       <c r="R8" s="48"/>
       <c r="S8" s="48"/>
       <c r="T8" s="48"/>
-      <c r="U8" s="106"/>
+      <c r="U8" s="109"/>
     </row>
     <row r="9" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -3591,25 +3590,25 @@
         <f t="shared" si="2"/>
         <v>700</v>
       </c>
-      <c r="N26" s="113" t="s">
+      <c r="N26" s="103" t="s">
         <v>209</v>
       </c>
-      <c r="O26" s="113" t="s">
+      <c r="O26" s="103" t="s">
         <v>209</v>
       </c>
-      <c r="P26" s="113" t="s">
+      <c r="P26" s="103" t="s">
         <v>209</v>
       </c>
-      <c r="Q26" s="113" t="s">
+      <c r="Q26" s="103" t="s">
         <v>209</v>
       </c>
-      <c r="R26" s="113" t="s">
+      <c r="R26" s="103" t="s">
         <v>209</v>
       </c>
-      <c r="S26" s="113" t="s">
+      <c r="S26" s="103" t="s">
         <v>209</v>
       </c>
-      <c r="T26" s="113" t="s">
+      <c r="T26" s="103" t="s">
         <v>209</v>
       </c>
       <c r="U26" s="34"/>
@@ -5664,11 +5663,11 @@
       <c r="L58" s="80"/>
       <c r="M58" s="80"/>
       <c r="N58" s="81"/>
-      <c r="O58" s="103" t="s">
+      <c r="O58" s="106" t="s">
         <v>288</v>
       </c>
-      <c r="P58" s="104"/>
-      <c r="Q58" s="104"/>
+      <c r="P58" s="107"/>
+      <c r="Q58" s="107"/>
       <c r="R58" s="94">
         <f>SUM(R10:R57)</f>
         <v>267.60030000000012</v>
@@ -5697,11 +5696,11 @@
       <c r="L59" s="39"/>
       <c r="M59" s="39"/>
       <c r="N59" s="82"/>
-      <c r="O59" s="109" t="s">
+      <c r="O59" s="112" t="s">
         <v>289</v>
       </c>
-      <c r="P59" s="110"/>
-      <c r="Q59" s="110"/>
+      <c r="P59" s="113"/>
+      <c r="Q59" s="113"/>
       <c r="R59" s="95">
         <f>R58/10</f>
         <v>26.760030000000011</v>
@@ -5714,11 +5713,11 @@
       <c r="U59" s="92"/>
     </row>
     <row r="60" spans="1:21" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="O60" s="103" t="s">
+      <c r="O60" s="106" t="s">
         <v>287</v>
       </c>
-      <c r="P60" s="104"/>
-      <c r="Q60" s="104"/>
+      <c r="P60" s="107"/>
+      <c r="Q60" s="107"/>
       <c r="R60" s="95">
         <v>15.6</v>
       </c>
@@ -5729,11 +5728,11 @@
       <c r="U60" s="92"/>
     </row>
     <row r="61" spans="1:21" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="O61" s="103" t="s">
+      <c r="O61" s="106" t="s">
         <v>290</v>
       </c>
-      <c r="P61" s="104"/>
-      <c r="Q61" s="104"/>
+      <c r="P61" s="107"/>
+      <c r="Q61" s="107"/>
       <c r="R61" s="96">
         <f>SUM(R59:R60)</f>
         <v>42.360030000000009</v>
@@ -5756,51 +5755,51 @@
     <mergeCell ref="O59:Q59"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="P30" r:id="rId1" xr:uid="{2F7ACCE1-6330-4FB8-8E97-307E3319C2DE}"/>
-    <hyperlink ref="P10" r:id="rId2" xr:uid="{2FD930C5-FD4D-4485-90FD-8F42F2FB86D7}"/>
-    <hyperlink ref="P11" r:id="rId3" xr:uid="{688A594C-DCDB-431E-8DB2-3B73EB820898}"/>
-    <hyperlink ref="P12" r:id="rId4" xr:uid="{6BEA14D3-818D-4150-AAF2-C8F29C4E446F}"/>
-    <hyperlink ref="P13" r:id="rId5" xr:uid="{3BC620E1-E1C4-4CB2-97F8-0D7A99A20BA6}"/>
-    <hyperlink ref="P14" r:id="rId6" xr:uid="{86CA8042-2DC3-473D-A979-72AA83514D52}"/>
-    <hyperlink ref="P15" r:id="rId7" xr:uid="{10F67B99-3057-42AF-9D42-570C3F0C60F9}"/>
-    <hyperlink ref="P16" r:id="rId8" xr:uid="{C60F0072-FB12-4DC1-A5ED-163CB541B5EE}"/>
-    <hyperlink ref="P17" r:id="rId9" xr:uid="{D6325761-9FC1-40D8-A82A-BE2228F64DD4}"/>
-    <hyperlink ref="P18" r:id="rId10" xr:uid="{FB501BA7-9DA3-4FB5-96C5-5C3DE4D94636}"/>
-    <hyperlink ref="P19" r:id="rId11" xr:uid="{52A5DA0D-4027-4FB3-9D9D-CCAE0B3978E9}"/>
-    <hyperlink ref="P20" r:id="rId12" xr:uid="{A040D7AB-FCEA-42F9-AA19-32A18DFCC9FD}"/>
-    <hyperlink ref="P21" r:id="rId13" xr:uid="{78C6F96A-EC11-4F4D-BEC2-D9CE6B61E957}"/>
-    <hyperlink ref="P22" r:id="rId14" xr:uid="{DCE2F2B0-D3E6-44CA-918D-195765810164}"/>
-    <hyperlink ref="P24" r:id="rId15" xr:uid="{EFF8AB1D-F8FF-44D4-AD07-A2579EB1243B}"/>
-    <hyperlink ref="P25" r:id="rId16" xr:uid="{01F791E4-771A-4DD8-A4EF-F9126473CB59}"/>
-    <hyperlink ref="P28" r:id="rId17" xr:uid="{BBAB8A3F-1C1F-4113-8688-4EF88392549D}"/>
-    <hyperlink ref="P29" r:id="rId18" xr:uid="{211E7481-A001-46F9-BD5F-2A77B5800AB3}"/>
-    <hyperlink ref="P32" r:id="rId19" xr:uid="{7CDD01B6-C01F-461B-9592-D9BA3EA621F2}"/>
-    <hyperlink ref="P33" r:id="rId20" xr:uid="{062A632F-F1EB-4EB4-9D86-5BE7FA6F6DEB}"/>
-    <hyperlink ref="P34" r:id="rId21" xr:uid="{E7F7B3C8-9A79-4316-957C-7140C5ACF4B9}"/>
-    <hyperlink ref="P35" r:id="rId22" xr:uid="{1E45DDAB-804E-4CC3-BD40-0EBB99F81712}"/>
-    <hyperlink ref="P37" r:id="rId23" xr:uid="{89232A72-9254-4A2F-8534-FB7B74758559}"/>
-    <hyperlink ref="P38" r:id="rId24" xr:uid="{3948AA46-8D94-453A-969E-5BE874AF0204}"/>
-    <hyperlink ref="P39" r:id="rId25" xr:uid="{166ADBD4-943F-4ECC-95E2-D4E57A9202DA}"/>
-    <hyperlink ref="P40" r:id="rId26" xr:uid="{4131DE7B-77EF-497B-932D-D11A51BAFAD8}"/>
-    <hyperlink ref="P41" r:id="rId27" xr:uid="{EE42F985-F887-481A-ABAD-3892E9DF1783}"/>
-    <hyperlink ref="P42" r:id="rId28" xr:uid="{4723D86B-1885-45F4-8D16-D3E5F7BACAEA}"/>
-    <hyperlink ref="P43" r:id="rId29" xr:uid="{50402008-E888-42E5-B37B-4C1CA46E922C}"/>
-    <hyperlink ref="P44" r:id="rId30" xr:uid="{02C490EA-37FA-4E68-A4A5-44A8D3ED5B48}"/>
-    <hyperlink ref="P46" r:id="rId31" xr:uid="{1EF6C760-C341-401C-9175-F7D45AC47B77}"/>
-    <hyperlink ref="P47" r:id="rId32" xr:uid="{591682BE-520A-4F3D-8A8A-ABC5F9E8F6DE}"/>
-    <hyperlink ref="P48" r:id="rId33" xr:uid="{99988462-F1C8-44B4-96C3-1B88F5BF930D}"/>
-    <hyperlink ref="P49" r:id="rId34" xr:uid="{775129CE-5F45-483A-BA6C-9CDD4367CEB5}"/>
-    <hyperlink ref="P50" r:id="rId35" xr:uid="{5659A1E3-D32B-4B55-87D4-9B5A95CCA83F}"/>
-    <hyperlink ref="P51" r:id="rId36" xr:uid="{0E564FE6-FFFB-4AFD-AE93-4B98F9805F61}"/>
-    <hyperlink ref="P52" r:id="rId37" xr:uid="{D03B4D86-7CD8-4450-BC82-487F997A38AB}"/>
-    <hyperlink ref="P53" r:id="rId38" xr:uid="{C6B26088-BEA0-4425-9AF3-1A2B5444A64E}"/>
-    <hyperlink ref="P54" r:id="rId39" xr:uid="{B0F6DBA4-47C8-421E-8D8D-E7CDDAA9B8E7}"/>
-    <hyperlink ref="P55" r:id="rId40" xr:uid="{845F5956-7C23-4391-9FD5-6E93246239D6}"/>
-    <hyperlink ref="P56" r:id="rId41" xr:uid="{2EF96914-BBAD-4919-B0A3-9757DF18FBAA}"/>
-    <hyperlink ref="P57" r:id="rId42" xr:uid="{6BD0D022-CC4B-4A90-956C-EA7C7D09A4BB}"/>
-    <hyperlink ref="P27" r:id="rId43" xr:uid="{6F20BBBA-327D-49D2-8651-44DD5479D4F7}"/>
-    <hyperlink ref="P23" r:id="rId44" xr:uid="{9A445BA4-E19F-4F79-9207-C31C95F96585}"/>
-    <hyperlink ref="P36" r:id="rId45" xr:uid="{3128E03B-1874-41DC-B355-5921D175B75E}"/>
+    <hyperlink ref="P30" r:id="rId1"/>
+    <hyperlink ref="P10" r:id="rId2"/>
+    <hyperlink ref="P11" r:id="rId3"/>
+    <hyperlink ref="P12" r:id="rId4"/>
+    <hyperlink ref="P13" r:id="rId5"/>
+    <hyperlink ref="P14" r:id="rId6"/>
+    <hyperlink ref="P15" r:id="rId7"/>
+    <hyperlink ref="P16" r:id="rId8"/>
+    <hyperlink ref="P17" r:id="rId9"/>
+    <hyperlink ref="P18" r:id="rId10"/>
+    <hyperlink ref="P19" r:id="rId11"/>
+    <hyperlink ref="P20" r:id="rId12"/>
+    <hyperlink ref="P21" r:id="rId13"/>
+    <hyperlink ref="P22" r:id="rId14"/>
+    <hyperlink ref="P24" r:id="rId15"/>
+    <hyperlink ref="P25" r:id="rId16"/>
+    <hyperlink ref="P28" r:id="rId17"/>
+    <hyperlink ref="P29" r:id="rId18"/>
+    <hyperlink ref="P32" r:id="rId19"/>
+    <hyperlink ref="P33" r:id="rId20"/>
+    <hyperlink ref="P34" r:id="rId21"/>
+    <hyperlink ref="P35" r:id="rId22"/>
+    <hyperlink ref="P37" r:id="rId23"/>
+    <hyperlink ref="P38" r:id="rId24"/>
+    <hyperlink ref="P39" r:id="rId25"/>
+    <hyperlink ref="P40" r:id="rId26"/>
+    <hyperlink ref="P41" r:id="rId27"/>
+    <hyperlink ref="P42" r:id="rId28"/>
+    <hyperlink ref="P43" r:id="rId29"/>
+    <hyperlink ref="P44" r:id="rId30"/>
+    <hyperlink ref="P46" r:id="rId31"/>
+    <hyperlink ref="P47" r:id="rId32"/>
+    <hyperlink ref="P48" r:id="rId33"/>
+    <hyperlink ref="P49" r:id="rId34"/>
+    <hyperlink ref="P50" r:id="rId35"/>
+    <hyperlink ref="P51" r:id="rId36"/>
+    <hyperlink ref="P52" r:id="rId37"/>
+    <hyperlink ref="P53" r:id="rId38"/>
+    <hyperlink ref="P54" r:id="rId39"/>
+    <hyperlink ref="P55" r:id="rId40"/>
+    <hyperlink ref="P56" r:id="rId41"/>
+    <hyperlink ref="P57" r:id="rId42"/>
+    <hyperlink ref="P27" r:id="rId43"/>
+    <hyperlink ref="P23" r:id="rId44"/>
+    <hyperlink ref="P36" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId46"/>

</xml_diff>

<commit_message>
Quotation added in LCSC BOM for part num 22232111 #1
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Bill of Materials-John_Main.xlsx
+++ b/Deliverables/BOM/Bill of Materials-John_Main.xlsx
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="302">
   <si>
     <t>Component list</t>
   </si>
@@ -917,9 +917,6 @@
   </si>
   <si>
     <t xml:space="preserve">Custom Supplier </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Urooj Is part Custom supplier se Quotation le len </t>
   </si>
   <si>
     <t>R12, R19, R20, R25, R26, RF3</t>
@@ -3919,19 +3916,21 @@
       <c r="P31" s="32" t="s">
         <v>295</v>
       </c>
-      <c r="Q31" s="37"/>
+      <c r="Q31" s="37">
+        <v>0.83</v>
+      </c>
       <c r="R31" s="38">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="S31" s="37"/>
+        <v>18.259999999999998</v>
+      </c>
+      <c r="S31" s="37">
+        <v>0.83</v>
+      </c>
       <c r="T31" s="38">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="U31" s="100" t="s">
-        <v>296</v>
-      </c>
+        <v>170.15</v>
+      </c>
+      <c r="U31" s="100"/>
     </row>
     <row r="32" spans="1:21" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
@@ -4138,7 +4137,7 @@
         <v>26</v>
       </c>
       <c r="C35" s="44" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D35" s="44" t="s">
         <v>79</v>
@@ -4203,25 +4202,25 @@
         <v>27</v>
       </c>
       <c r="C36" s="44" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D36" s="44" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E36" s="44" t="s">
         <v>116</v>
       </c>
       <c r="F36" s="60" t="s">
+        <v>299</v>
+      </c>
+      <c r="G36" s="69" t="s">
         <v>300</v>
-      </c>
-      <c r="G36" s="69" t="s">
-        <v>301</v>
       </c>
       <c r="H36" s="64" t="s">
         <v>156</v>
       </c>
       <c r="I36" s="44" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J36" s="64" t="s">
         <v>191</v>
@@ -5670,12 +5669,12 @@
       <c r="Q58" s="107"/>
       <c r="R58" s="94">
         <f>SUM(R10:R57)</f>
-        <v>267.60030000000012</v>
+        <v>285.86030000000017</v>
       </c>
       <c r="S58" s="97"/>
       <c r="T58" s="94">
         <f>SUM(T10:T57)</f>
-        <v>1828.809</v>
+        <v>1998.9589999999998</v>
       </c>
       <c r="U58" s="91"/>
     </row>
@@ -5703,12 +5702,12 @@
       <c r="Q59" s="113"/>
       <c r="R59" s="95">
         <f>R58/10</f>
-        <v>26.760030000000011</v>
+        <v>28.586030000000015</v>
       </c>
       <c r="S59" s="98"/>
       <c r="T59" s="95">
         <f>T58/100</f>
-        <v>18.28809</v>
+        <v>19.98959</v>
       </c>
       <c r="U59" s="92"/>
     </row>
@@ -5735,12 +5734,12 @@
       <c r="Q61" s="107"/>
       <c r="R61" s="96">
         <f>SUM(R59:R60)</f>
-        <v>42.360030000000009</v>
+        <v>44.186030000000017</v>
       </c>
       <c r="S61" s="99"/>
       <c r="T61" s="96">
         <f>SUM(T59:T60)</f>
-        <v>102.58808999999999</v>
+        <v>104.28959</v>
       </c>
       <c r="U61" s="93"/>
     </row>

</xml_diff>